<commit_message>
fix: update existing API
</commit_message>
<xml_diff>
--- a/luutru-prototypes/danh-sach-chuc-nang-storage.xlsx
+++ b/luutru-prototypes/danh-sach-chuc-nang-storage.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Personal\Study\Personal\Viettel\intern\cloud-drive\luutru-prototypes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAD4D11D-A597-47AB-8964-F10230738C6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81B8DFD0-A95D-4DFF-A2AB-F7CD8476AB51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="186">
   <si>
     <t>CHỨC NĂNG CẦN TRIỂN KHAI — NGƯỜI DÙNG</t>
   </si>
@@ -590,6 +590,9 @@
   </si>
   <si>
     <t>Hoàn thành</t>
+  </si>
+  <si>
+    <t>Chưa bắt đầu</t>
   </si>
 </sst>
 </file>
@@ -1219,7 +1222,7 @@
         <v>22</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F12" s="9"/>
     </row>
@@ -1237,7 +1240,7 @@
         <v>24</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F13" s="9"/>
     </row>

</xml_diff>